<commit_message>
Cyclopean: per-footing detail of excavation before/after, cyclopean layer and backfill
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/cyclopean.xlsx
+++ b/cyclopean.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cyclopean" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Footings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Detail (offset from hatch)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Detail (offset from concrete)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cyclopean" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Footings" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -59,10 +61,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,8 +433,634 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Area 2 hatched footings - excavation 1120.9 -&gt; 1118.0 (2.9 m), cyclopean 0.5 m (1118.0 -&gt; 1117.5); offset 1.0 m from the hatch (blinding) outline; no offset on the retaining-wall outer face</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="62" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Footing</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Blinding area (m²)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Cyclopean area (m²)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Offset band (m²)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Excavation before - blinding x 2.9 (m³)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Excavation after - cyclopean x 2.9 (m³)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Difference to 1118 (m³)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Cyclopean layer excavation x 0.5 (m³)</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Total extra excavation (m³)</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Cyclopean concrete (m³)</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Extra backfill - band x 2.9 (m³)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Retaining-wall footing - north/east part</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>180.09</v>
+      </c>
+      <c r="C4" t="n">
+        <v>262.24</v>
+      </c>
+      <c r="D4" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="E4" t="n">
+        <v>522.25</v>
+      </c>
+      <c r="F4" t="n">
+        <v>760.49</v>
+      </c>
+      <c r="G4" t="n">
+        <v>238.23</v>
+      </c>
+      <c r="H4" t="n">
+        <v>131.12</v>
+      </c>
+      <c r="I4" t="n">
+        <v>369.35</v>
+      </c>
+      <c r="J4" t="n">
+        <v>131.12</v>
+      </c>
+      <c r="K4" t="n">
+        <v>238.23</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Retaining-wall footing - south/curve part</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>38.65</v>
+      </c>
+      <c r="C5" t="n">
+        <v>60.51</v>
+      </c>
+      <c r="D5" t="n">
+        <v>21.87</v>
+      </c>
+      <c r="E5" t="n">
+        <v>112.07</v>
+      </c>
+      <c r="F5" t="n">
+        <v>175.48</v>
+      </c>
+      <c r="G5" t="n">
+        <v>63.41</v>
+      </c>
+      <c r="H5" t="n">
+        <v>30.26</v>
+      </c>
+      <c r="I5" t="n">
+        <v>93.67</v>
+      </c>
+      <c r="J5" t="n">
+        <v>30.26</v>
+      </c>
+      <c r="K5" t="n">
+        <v>63.41</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pad footing P1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>14.44</v>
+      </c>
+      <c r="C6" t="n">
+        <v>29.95</v>
+      </c>
+      <c r="D6" t="n">
+        <v>15.51</v>
+      </c>
+      <c r="E6" t="n">
+        <v>41.88</v>
+      </c>
+      <c r="F6" t="n">
+        <v>86.84</v>
+      </c>
+      <c r="G6" t="n">
+        <v>44.97</v>
+      </c>
+      <c r="H6" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="I6" t="n">
+        <v>59.94</v>
+      </c>
+      <c r="J6" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="K6" t="n">
+        <v>44.97</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pad footing P2</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="C7" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="E7" t="n">
+        <v>15.23</v>
+      </c>
+      <c r="F7" t="n">
+        <v>51.42</v>
+      </c>
+      <c r="G7" t="n">
+        <v>36.19</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8.869999999999999</v>
+      </c>
+      <c r="I7" t="n">
+        <v>45.06</v>
+      </c>
+      <c r="J7" t="n">
+        <v>8.869999999999999</v>
+      </c>
+      <c r="K7" t="n">
+        <v>36.19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pad footing P3</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="C8" t="n">
+        <v>13.82</v>
+      </c>
+      <c r="D8" t="n">
+        <v>8.57</v>
+      </c>
+      <c r="E8" t="n">
+        <v>15.23</v>
+      </c>
+      <c r="F8" t="n">
+        <v>40.07</v>
+      </c>
+      <c r="G8" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="H8" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="I8" t="n">
+        <v>31.76</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="K8" t="n">
+        <v>24.85</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>243.67</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>384.24</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>140.57</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>706.65</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>1114.3</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>407.65</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>192.12</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>599.77</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>192.12</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>407.65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Area 2 hatched footings - excavation 1120.9 -&gt; 1118.0 (2.9 m), cyclopean 0.5 m (1118.0 -&gt; 1117.5); offset 1.0 m from the concrete face (0.9 m from the hatch); no offset on the retaining-wall outer face</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="62" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Footing</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Blinding area (m²)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Cyclopean area (m²)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Offset band (m²)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Excavation before - blinding x 2.9 (m³)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Excavation after - cyclopean x 2.9 (m³)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Difference to 1118 (m³)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Cyclopean layer excavation x 0.5 (m³)</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Total extra excavation (m³)</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Cyclopean concrete (m³)</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Extra backfill - band x 2.9 (m³)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Retaining-wall footing - north/east part</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>180.09</v>
+      </c>
+      <c r="C4" t="n">
+        <v>254</v>
+      </c>
+      <c r="D4" t="n">
+        <v>73.91</v>
+      </c>
+      <c r="E4" t="n">
+        <v>522.25</v>
+      </c>
+      <c r="F4" t="n">
+        <v>736.6</v>
+      </c>
+      <c r="G4" t="n">
+        <v>214.35</v>
+      </c>
+      <c r="H4" t="n">
+        <v>127</v>
+      </c>
+      <c r="I4" t="n">
+        <v>341.35</v>
+      </c>
+      <c r="J4" t="n">
+        <v>127</v>
+      </c>
+      <c r="K4" t="n">
+        <v>214.35</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Retaining-wall footing - south/curve part</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>38.65</v>
+      </c>
+      <c r="C5" t="n">
+        <v>58.35</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="E5" t="n">
+        <v>112.07</v>
+      </c>
+      <c r="F5" t="n">
+        <v>169.21</v>
+      </c>
+      <c r="G5" t="n">
+        <v>57.13</v>
+      </c>
+      <c r="H5" t="n">
+        <v>29.17</v>
+      </c>
+      <c r="I5" t="n">
+        <v>86.31</v>
+      </c>
+      <c r="J5" t="n">
+        <v>29.17</v>
+      </c>
+      <c r="K5" t="n">
+        <v>57.13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pad footing P1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>14.44</v>
+      </c>
+      <c r="C6" t="n">
+        <v>28.33</v>
+      </c>
+      <c r="D6" t="n">
+        <v>13.89</v>
+      </c>
+      <c r="E6" t="n">
+        <v>41.88</v>
+      </c>
+      <c r="F6" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="G6" t="n">
+        <v>40.28</v>
+      </c>
+      <c r="H6" t="n">
+        <v>14.16</v>
+      </c>
+      <c r="I6" t="n">
+        <v>54.44</v>
+      </c>
+      <c r="J6" t="n">
+        <v>14.16</v>
+      </c>
+      <c r="K6" t="n">
+        <v>40.28</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pad footing P2</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="C7" t="n">
+        <v>16.29</v>
+      </c>
+      <c r="D7" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="E7" t="n">
+        <v>15.23</v>
+      </c>
+      <c r="F7" t="n">
+        <v>47.24</v>
+      </c>
+      <c r="G7" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="I7" t="n">
+        <v>40.16</v>
+      </c>
+      <c r="J7" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="K7" t="n">
+        <v>32.01</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pad footing P3</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="C8" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="D8" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="E8" t="n">
+        <v>15.23</v>
+      </c>
+      <c r="F8" t="n">
+        <v>37.33</v>
+      </c>
+      <c r="G8" t="n">
+        <v>22.11</v>
+      </c>
+      <c r="H8" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="I8" t="n">
+        <v>28.54</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="K8" t="n">
+        <v>22.11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>243.67</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>369.84</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>126.17</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>706.65</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>1072.53</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>365.88</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>184.92</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>550.8</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>184.92</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>365.88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -630,7 +1261,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Cyclopean between 1118.0 and 1118.5 (no excavation below 1118); backfill from 1118.5
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/cyclopean.xlsx
+++ b/cyclopean.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -445,14 +445,12 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Area 2 hatched footings - excavation 1120.9 -&gt; 1118.0 (2.9 m), cyclopean 0.5 m (1118.0 -&gt; 1117.5); offset 1.0 m from the hatch (blinding) outline; no offset on the retaining-wall outer face</t>
+          <t>Area 2 hatched footings - excavation 1120.9 -&gt; 1118.0 (2.9 m), cyclopean 0.5 m (1118.0 -&gt; 1118.5, footings on top at 1118.5); offset 1.0 m from the hatch (blinding) outline; no offset on the retaining-wall outer face</t>
         </is>
       </c>
     </row>
@@ -489,27 +487,17 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Difference to 1118 (m³)</t>
+          <t>Extra excavation = difference to 1118 (m³)</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Cyclopean layer excavation x 0.5 (m³)</t>
+          <t>Cyclopean concrete (m³)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Total extra excavation (m³)</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Cyclopean concrete (m³)</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Extra backfill - band x 2.9 (m³)</t>
+          <t>Extra backfill - band x 2.4 (1118.5 -&gt; 1120.9) (m³)</t>
         </is>
       </c>
     </row>
@@ -541,13 +529,7 @@
         <v>131.12</v>
       </c>
       <c r="I4" t="n">
-        <v>369.35</v>
-      </c>
-      <c r="J4" t="n">
-        <v>131.12</v>
-      </c>
-      <c r="K4" t="n">
-        <v>238.23</v>
+        <v>197.16</v>
       </c>
     </row>
     <row r="5">
@@ -578,13 +560,7 @@
         <v>30.26</v>
       </c>
       <c r="I5" t="n">
-        <v>93.67</v>
-      </c>
-      <c r="J5" t="n">
-        <v>30.26</v>
-      </c>
-      <c r="K5" t="n">
-        <v>63.41</v>
+        <v>52.48</v>
       </c>
     </row>
     <row r="6">
@@ -615,13 +591,7 @@
         <v>14.97</v>
       </c>
       <c r="I6" t="n">
-        <v>59.94</v>
-      </c>
-      <c r="J6" t="n">
-        <v>14.97</v>
-      </c>
-      <c r="K6" t="n">
-        <v>44.97</v>
+        <v>37.21</v>
       </c>
     </row>
     <row r="7">
@@ -652,13 +622,7 @@
         <v>8.869999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>45.06</v>
-      </c>
-      <c r="J7" t="n">
-        <v>8.869999999999999</v>
-      </c>
-      <c r="K7" t="n">
-        <v>36.19</v>
+        <v>29.95</v>
       </c>
     </row>
     <row r="8">
@@ -689,13 +653,7 @@
         <v>6.91</v>
       </c>
       <c r="I8" t="n">
-        <v>31.76</v>
-      </c>
-      <c r="J8" t="n">
-        <v>6.91</v>
-      </c>
-      <c r="K8" t="n">
-        <v>24.85</v>
+        <v>20.56</v>
       </c>
     </row>
     <row r="9">
@@ -726,13 +684,7 @@
         <v>192.12</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>599.77</v>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>192.12</v>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>407.65</v>
+        <v>337.37</v>
       </c>
     </row>
   </sheetData>
@@ -746,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -758,14 +710,12 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Area 2 hatched footings - excavation 1120.9 -&gt; 1118.0 (2.9 m), cyclopean 0.5 m (1118.0 -&gt; 1117.5); offset 1.0 m from the concrete face (0.9 m from the hatch); no offset on the retaining-wall outer face</t>
+          <t>Area 2 hatched footings - excavation 1120.9 -&gt; 1118.0 (2.9 m), cyclopean 0.5 m (1118.0 -&gt; 1118.5, footings on top at 1118.5); offset 1.0 m from the concrete face (0.9 m from the hatch); no offset on the retaining-wall outer face</t>
         </is>
       </c>
     </row>
@@ -802,27 +752,17 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Difference to 1118 (m³)</t>
+          <t>Extra excavation = difference to 1118 (m³)</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Cyclopean layer excavation x 0.5 (m³)</t>
+          <t>Cyclopean concrete (m³)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Total extra excavation (m³)</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Cyclopean concrete (m³)</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Extra backfill - band x 2.9 (m³)</t>
+          <t>Extra backfill - band x 2.4 (1118.5 -&gt; 1120.9) (m³)</t>
         </is>
       </c>
     </row>
@@ -854,13 +794,7 @@
         <v>127</v>
       </c>
       <c r="I4" t="n">
-        <v>341.35</v>
-      </c>
-      <c r="J4" t="n">
-        <v>127</v>
-      </c>
-      <c r="K4" t="n">
-        <v>214.35</v>
+        <v>177.39</v>
       </c>
     </row>
     <row r="5">
@@ -891,13 +825,7 @@
         <v>29.17</v>
       </c>
       <c r="I5" t="n">
-        <v>86.31</v>
-      </c>
-      <c r="J5" t="n">
-        <v>29.17</v>
-      </c>
-      <c r="K5" t="n">
-        <v>57.13</v>
+        <v>47.28</v>
       </c>
     </row>
     <row r="6">
@@ -928,13 +856,7 @@
         <v>14.16</v>
       </c>
       <c r="I6" t="n">
-        <v>54.44</v>
-      </c>
-      <c r="J6" t="n">
-        <v>14.16</v>
-      </c>
-      <c r="K6" t="n">
-        <v>40.28</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="7">
@@ -965,13 +887,7 @@
         <v>8.140000000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>40.16</v>
-      </c>
-      <c r="J7" t="n">
-        <v>8.140000000000001</v>
-      </c>
-      <c r="K7" t="n">
-        <v>32.01</v>
+        <v>26.49</v>
       </c>
     </row>
     <row r="8">
@@ -1002,13 +918,7 @@
         <v>6.44</v>
       </c>
       <c r="I8" t="n">
-        <v>28.54</v>
-      </c>
-      <c r="J8" t="n">
-        <v>6.44</v>
-      </c>
-      <c r="K8" t="n">
-        <v>22.11</v>
+        <v>18.29</v>
       </c>
     </row>
     <row r="9">
@@ -1039,13 +949,7 @@
         <v>184.92</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>550.8</v>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>184.92</v>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>365.88</v>
+        <v>302.8</v>
       </c>
     </row>
   </sheetData>
@@ -1059,7 +963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -1125,7 +1029,7 @@
         <v>1118</v>
       </c>
       <c r="D3" t="n">
-        <v>1117.5</v>
+        <v>1118.5</v>
       </c>
       <c r="E3" t="n">
         <v>0.5</v>
@@ -1149,110 +1053,88 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1) Cyclopean layer under the footings</t>
+          <t>Widening the pits by the offset band</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>384.24</v>
+        <v>140.57</v>
       </c>
       <c r="C6" t="n">
+        <v>1120.9</v>
+      </c>
+      <c r="D6" t="n">
         <v>1118</v>
       </c>
-      <c r="D6" t="n">
-        <v>1117.5</v>
-      </c>
       <c r="E6" t="n">
-        <v>0.5</v>
+        <v>2.900000000000091</v>
       </c>
       <c r="F6" t="n">
-        <v>192.12</v>
+        <v>407.65</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2) Widening the pits by the offset band</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>140.57</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1120.9</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1118</v>
-      </c>
-      <c r="E7" t="n">
-        <v>2.900000000000091</v>
-      </c>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Total extra excavation</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
         <v>407.65</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Total extra excavation</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="n">
-        <v>599.77</v>
-      </c>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>EXTRA BACKFILL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>EXTRA BACKFILL</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Offset band above the cyclopean</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B10" t="n">
         <v>140.57</v>
       </c>
-      <c r="C11" t="n">
-        <v>1118</v>
-      </c>
-      <c r="D11" t="n">
+      <c r="C10" t="n">
+        <v>1118.5</v>
+      </c>
+      <c r="D10" t="n">
         <v>1120.9</v>
       </c>
-      <c r="E11" t="n">
-        <v>2.900000000000091</v>
-      </c>
-      <c r="F11" t="n">
-        <v>407.65</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="E10" t="n">
+        <v>2.400000000000091</v>
+      </c>
+      <c r="F10" t="n">
+        <v>337.37</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Check - offset 1 m from the concrete face (0.9 m from the hatch)</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B12" t="n">
         <v>369.84</v>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="n">
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
         <v>0.5</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F12" t="n">
         <v>184.92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Cyclopean: adopt 1 m offset from the concrete face (hatch offset kept as alternative)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/cyclopean.xlsx
+++ b/cyclopean.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Detail (offset from hatch)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Detail (offset from concrete)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Detail (offset from concrete)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Detail (offset from hatch)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Cyclopean" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Footings" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -450,7 +450,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Area 2 hatched footings - excavation 1120.9 -&gt; 1118.0 (2.9 m), cyclopean 0.5 m (1118.0 -&gt; 1118.5, footings on top at 1118.5); offset 1.0 m from the hatch (blinding) outline; no offset on the retaining-wall outer face</t>
+          <t>Area 2 hatched footings - excavation 1120.9 -&gt; 1118.0 (2.9 m), cyclopean 0.5 m (1118.0 -&gt; 1118.5, footings on top at 1118.5); offset 1.0 m from the concrete face (0.9 m from the hatch); no offset on the retaining-wall outer face</t>
         </is>
       </c>
     </row>
@@ -511,25 +511,25 @@
         <v>180.09</v>
       </c>
       <c r="C4" t="n">
-        <v>262.24</v>
+        <v>254</v>
       </c>
       <c r="D4" t="n">
-        <v>82.15000000000001</v>
+        <v>73.91</v>
       </c>
       <c r="E4" t="n">
         <v>522.25</v>
       </c>
       <c r="F4" t="n">
-        <v>760.49</v>
+        <v>736.6</v>
       </c>
       <c r="G4" t="n">
-        <v>238.23</v>
+        <v>214.35</v>
       </c>
       <c r="H4" t="n">
-        <v>131.12</v>
+        <v>127</v>
       </c>
       <c r="I4" t="n">
-        <v>197.16</v>
+        <v>177.39</v>
       </c>
     </row>
     <row r="5">
@@ -542,25 +542,25 @@
         <v>38.65</v>
       </c>
       <c r="C5" t="n">
-        <v>60.51</v>
+        <v>58.35</v>
       </c>
       <c r="D5" t="n">
-        <v>21.87</v>
+        <v>19.7</v>
       </c>
       <c r="E5" t="n">
         <v>112.07</v>
       </c>
       <c r="F5" t="n">
-        <v>175.48</v>
+        <v>169.21</v>
       </c>
       <c r="G5" t="n">
-        <v>63.41</v>
+        <v>57.13</v>
       </c>
       <c r="H5" t="n">
-        <v>30.26</v>
+        <v>29.17</v>
       </c>
       <c r="I5" t="n">
-        <v>52.48</v>
+        <v>47.28</v>
       </c>
     </row>
     <row r="6">
@@ -573,25 +573,25 @@
         <v>14.44</v>
       </c>
       <c r="C6" t="n">
-        <v>29.95</v>
+        <v>28.33</v>
       </c>
       <c r="D6" t="n">
-        <v>15.51</v>
+        <v>13.89</v>
       </c>
       <c r="E6" t="n">
         <v>41.88</v>
       </c>
       <c r="F6" t="n">
-        <v>86.84</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>44.97</v>
+        <v>40.28</v>
       </c>
       <c r="H6" t="n">
-        <v>14.97</v>
+        <v>14.16</v>
       </c>
       <c r="I6" t="n">
-        <v>37.21</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="7">
@@ -604,25 +604,25 @@
         <v>5.25</v>
       </c>
       <c r="C7" t="n">
-        <v>17.73</v>
+        <v>16.29</v>
       </c>
       <c r="D7" t="n">
-        <v>12.48</v>
+        <v>11.04</v>
       </c>
       <c r="E7" t="n">
         <v>15.23</v>
       </c>
       <c r="F7" t="n">
-        <v>51.42</v>
+        <v>47.24</v>
       </c>
       <c r="G7" t="n">
-        <v>36.19</v>
+        <v>32.01</v>
       </c>
       <c r="H7" t="n">
-        <v>8.869999999999999</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>29.95</v>
+        <v>26.49</v>
       </c>
     </row>
     <row r="8">
@@ -635,25 +635,25 @@
         <v>5.25</v>
       </c>
       <c r="C8" t="n">
-        <v>13.82</v>
+        <v>12.87</v>
       </c>
       <c r="D8" t="n">
-        <v>8.57</v>
+        <v>7.62</v>
       </c>
       <c r="E8" t="n">
         <v>15.23</v>
       </c>
       <c r="F8" t="n">
-        <v>40.07</v>
+        <v>37.33</v>
       </c>
       <c r="G8" t="n">
-        <v>24.85</v>
+        <v>22.11</v>
       </c>
       <c r="H8" t="n">
-        <v>6.91</v>
+        <v>6.44</v>
       </c>
       <c r="I8" t="n">
-        <v>20.56</v>
+        <v>18.29</v>
       </c>
     </row>
     <row r="9">
@@ -666,25 +666,25 @@
         <v>243.67</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>384.24</v>
+        <v>369.84</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>140.57</v>
+        <v>126.17</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>706.65</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1114.3</v>
+        <v>1072.53</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>407.65</v>
+        <v>365.88</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>192.12</v>
+        <v>184.92</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>337.37</v>
+        <v>302.8</v>
       </c>
     </row>
   </sheetData>
@@ -715,7 +715,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Area 2 hatched footings - excavation 1120.9 -&gt; 1118.0 (2.9 m), cyclopean 0.5 m (1118.0 -&gt; 1118.5, footings on top at 1118.5); offset 1.0 m from the concrete face (0.9 m from the hatch); no offset on the retaining-wall outer face</t>
+          <t>Area 2 hatched footings - excavation 1120.9 -&gt; 1118.0 (2.9 m), cyclopean 0.5 m (1118.0 -&gt; 1118.5, footings on top at 1118.5); offset 1.0 m from the hatch (blinding) outline; no offset on the retaining-wall outer face</t>
         </is>
       </c>
     </row>
@@ -776,25 +776,25 @@
         <v>180.09</v>
       </c>
       <c r="C4" t="n">
-        <v>254</v>
+        <v>262.24</v>
       </c>
       <c r="D4" t="n">
-        <v>73.91</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="E4" t="n">
         <v>522.25</v>
       </c>
       <c r="F4" t="n">
-        <v>736.6</v>
+        <v>760.49</v>
       </c>
       <c r="G4" t="n">
-        <v>214.35</v>
+        <v>238.23</v>
       </c>
       <c r="H4" t="n">
-        <v>127</v>
+        <v>131.12</v>
       </c>
       <c r="I4" t="n">
-        <v>177.39</v>
+        <v>197.16</v>
       </c>
     </row>
     <row r="5">
@@ -807,25 +807,25 @@
         <v>38.65</v>
       </c>
       <c r="C5" t="n">
-        <v>58.35</v>
+        <v>60.51</v>
       </c>
       <c r="D5" t="n">
-        <v>19.7</v>
+        <v>21.87</v>
       </c>
       <c r="E5" t="n">
         <v>112.07</v>
       </c>
       <c r="F5" t="n">
-        <v>169.21</v>
+        <v>175.48</v>
       </c>
       <c r="G5" t="n">
-        <v>57.13</v>
+        <v>63.41</v>
       </c>
       <c r="H5" t="n">
-        <v>29.17</v>
+        <v>30.26</v>
       </c>
       <c r="I5" t="n">
-        <v>47.28</v>
+        <v>52.48</v>
       </c>
     </row>
     <row r="6">
@@ -838,25 +838,25 @@
         <v>14.44</v>
       </c>
       <c r="C6" t="n">
-        <v>28.33</v>
+        <v>29.95</v>
       </c>
       <c r="D6" t="n">
-        <v>13.89</v>
+        <v>15.51</v>
       </c>
       <c r="E6" t="n">
         <v>41.88</v>
       </c>
       <c r="F6" t="n">
-        <v>82.15000000000001</v>
+        <v>86.84</v>
       </c>
       <c r="G6" t="n">
-        <v>40.28</v>
+        <v>44.97</v>
       </c>
       <c r="H6" t="n">
-        <v>14.16</v>
+        <v>14.97</v>
       </c>
       <c r="I6" t="n">
-        <v>33.33</v>
+        <v>37.21</v>
       </c>
     </row>
     <row r="7">
@@ -869,25 +869,25 @@
         <v>5.25</v>
       </c>
       <c r="C7" t="n">
-        <v>16.29</v>
+        <v>17.73</v>
       </c>
       <c r="D7" t="n">
-        <v>11.04</v>
+        <v>12.48</v>
       </c>
       <c r="E7" t="n">
         <v>15.23</v>
       </c>
       <c r="F7" t="n">
-        <v>47.24</v>
+        <v>51.42</v>
       </c>
       <c r="G7" t="n">
-        <v>32.01</v>
+        <v>36.19</v>
       </c>
       <c r="H7" t="n">
-        <v>8.140000000000001</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>26.49</v>
+        <v>29.95</v>
       </c>
     </row>
     <row r="8">
@@ -900,25 +900,25 @@
         <v>5.25</v>
       </c>
       <c r="C8" t="n">
-        <v>12.87</v>
+        <v>13.82</v>
       </c>
       <c r="D8" t="n">
-        <v>7.62</v>
+        <v>8.57</v>
       </c>
       <c r="E8" t="n">
         <v>15.23</v>
       </c>
       <c r="F8" t="n">
-        <v>37.33</v>
+        <v>40.07</v>
       </c>
       <c r="G8" t="n">
-        <v>22.11</v>
+        <v>24.85</v>
       </c>
       <c r="H8" t="n">
-        <v>6.44</v>
+        <v>6.91</v>
       </c>
       <c r="I8" t="n">
-        <v>18.29</v>
+        <v>20.56</v>
       </c>
     </row>
     <row r="9">
@@ -931,25 +931,25 @@
         <v>243.67</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>369.84</v>
+        <v>384.24</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>126.17</v>
+        <v>140.57</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>706.65</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1072.53</v>
+        <v>1114.3</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>365.88</v>
+        <v>407.65</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>184.92</v>
+        <v>192.12</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>302.8</v>
+        <v>337.37</v>
       </c>
     </row>
   </sheetData>
@@ -1019,11 +1019,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cyclopean concrete (footings + 1.0 m offset, flush on the retaining-wall outer face)</t>
+          <t>Cyclopean concrete (footings + 1.0 m offset from the concrete face, flush on the retaining-wall outer face)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>384.24</v>
+        <v>369.84</v>
       </c>
       <c r="C3" t="n">
         <v>1118</v>
@@ -1035,7 +1035,7 @@
         <v>0.5</v>
       </c>
       <c r="F3" t="n">
-        <v>192.12</v>
+        <v>184.92</v>
       </c>
     </row>
     <row r="5">
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>140.57</v>
+        <v>126.17</v>
       </c>
       <c r="C6" t="n">
         <v>1120.9</v>
@@ -1069,7 +1069,7 @@
         <v>2.900000000000091</v>
       </c>
       <c r="F6" t="n">
-        <v>407.65</v>
+        <v>365.88</v>
       </c>
     </row>
     <row r="7">
@@ -1083,7 +1083,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>407.65</v>
+        <v>365.88</v>
       </c>
     </row>
     <row r="9">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>140.57</v>
+        <v>126.17</v>
       </c>
       <c r="C10" t="n">
         <v>1118.5</v>
@@ -1117,17 +1117,17 @@
         <v>2.400000000000091</v>
       </c>
       <c r="F10" t="n">
-        <v>337.37</v>
+        <v>302.8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Check - offset 1 m from the concrete face (0.9 m from the hatch)</t>
+          <t>Alternative - offset 1 m from the hatch (blinding) outline</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>369.84</v>
+        <v>384.24</v>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
@@ -1135,7 +1135,7 @@
         <v>0.5</v>
       </c>
       <c r="F12" t="n">
-        <v>184.92</v>
+        <v>192.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>